<commit_message>
RESHIPPED (task124): loop 1 after the portal solve, the share among the unknown lines the targeted visits depleted decides; at $25.4 million a year RZ-10 Lakeview Terrace finishes in 2037 (whole-segment shares carried to the unknown lines 2038, every verification 2040)
Plan 4.3 now carries unknown lines at the share expected among the district's Lead Status Unknown lines; the whole-segment shares become a rung. Capital plan line $25.4 million, mobilisation $160,000, three zones' prices and two adjacent priority swaps for margins; ask files byte-identical to the loop-0 cut. Judge APPROVE (loop 1), leak reader clean on the final prompt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142Jt4Mt622iBfGoK24ivCU
</commit_message>
<xml_diff>
--- a/task124/golden/lslr_2027_programme.xlsx
+++ b/task124/golden/lslr_2027_programme.xlsx
@@ -22,9 +22,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="68">
-  <si>
-    <t>Every zone finished by 2037 at $27.1 million a year: lead service line replacement schedule, 2027 to 2037</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="75">
+  <si>
+    <t>Every zone finished by 2037 at $25.4 million a year: lead service line replacement schedule, 2027 to 2037</t>
   </si>
   <si>
     <t>Hollins Ford Regional Water District, LSLR programme office. Plan revision 2 zones in priority order; plan cost in 2027 dollars at the 2027 unit cost schedule. Prepared 11 January 2027 for the board meeting of 19 January 2027.</t>
@@ -96,79 +96,100 @@
     <t>Depot Square</t>
   </si>
   <si>
+    <t>RZ-03</t>
+  </si>
+  <si>
+    <t>Millrace</t>
+  </si>
+  <si>
     <t>RZ-12</t>
   </si>
   <si>
     <t>Kittering Village</t>
   </si>
   <si>
-    <t>RZ-03</t>
-  </si>
-  <si>
-    <t>Millrace</t>
-  </si>
-  <si>
     <t>RZ-08</t>
   </si>
   <si>
     <t>Elm Park</t>
   </si>
   <si>
+    <t>RZ-06</t>
+  </si>
+  <si>
+    <t>Wexley</t>
+  </si>
+  <si>
     <t>RZ-10</t>
   </si>
   <si>
     <t>Lakeview Terrace</t>
   </si>
   <si>
-    <t>RZ-06</t>
-  </si>
-  <si>
-    <t>Wexley</t>
-  </si>
-  <si>
     <t>All twelve zones</t>
   </si>
   <si>
-    <t>Last zone: RZ-06 Wexley, finished in programme year 2037, inside the 1 November 2037 deadline.</t>
-  </si>
-  <si>
-    <t>Lines to replace: the zone's Lead and GRR lines plus its Lead Status Unknown lines at the share found lead or GRR in their construction era on the segments verified whole (sheet Unknown-line shares).</t>
+    <t>Last zone: RZ-10 Lakeview Terrace, finished in programme year 2037, inside the 1 November 2037 deadline.</t>
+  </si>
+  <si>
+    <t>Lines to replace: the zone's Lead and GRR lines plus its Lead Status Unknown lines at the share of lead or GRR expected among the district's Lead Status Unknown lines of their construction era (plan 4.3; sheet Unknown-line shares).</t>
   </si>
   <si>
     <t>A zone is finished in the programme year in which the running total of the appropriation covers the running total of plan cost through it (plan 5.3). Lines rounded to the nearest ten and costs to the nearest $100,000; cumulative columns from unrounded zone costs.</t>
   </si>
   <si>
-    <t>Share of lines with no usable tap card expected to prove lead or GRR, by construction era</t>
-  </si>
-  <si>
-    <t>Lines with no usable tap card on the 78 main segments where every service line has been verified (each segment's lines exposed and verified together when its main was replaced, 2023 to 2026).</t>
+    <t>Share of the district's Lead Status Unknown lines expected to prove lead or GRR, by construction era</t>
+  </si>
+  <si>
+    <t>Lines built before 1989 with no usable tap card, all fourteen zones. Each is expected to prove lead or GRR at the share found on the 78 main segments where every service line has been verified (exposed together when the main was replaced, 2023 to 2026); the field verifications have already found part of that number, and the Lead Status Unknown lines carry the rest.</t>
   </si>
   <si>
     <t>Construction era</t>
   </si>
   <si>
+    <t>Lines with no usable tap card</t>
+  </si>
+  <si>
+    <t>Share on the segments verified whole</t>
+  </si>
+  <si>
+    <t>Expected to prove lead or GRR</t>
+  </si>
+  <si>
+    <t>Verified to date</t>
+  </si>
+  <si>
+    <t>Found lead or GRR</t>
+  </si>
+  <si>
+    <t>Lead Status Unknown</t>
+  </si>
+  <si>
+    <t>Expected lead or GRR among them</t>
+  </si>
+  <si>
+    <t>Share among Lead Status Unknown lines</t>
+  </si>
+  <si>
+    <t>Built before 1930</t>
+  </si>
+  <si>
+    <t>Built 1930 to 1949</t>
+  </si>
+  <si>
+    <t>Built 1950 to 1988</t>
+  </si>
+  <si>
+    <t>On the segments verified whole</t>
+  </si>
+  <si>
     <t>Lines verified</t>
   </si>
   <si>
-    <t>Found lead or GRR</t>
-  </si>
-  <si>
     <t>Share</t>
   </si>
   <si>
-    <t>Share across every verification (for comparison)</t>
-  </si>
-  <si>
-    <t>Built before 1930</t>
-  </si>
-  <si>
-    <t>Built 1930 to 1949</t>
-  </si>
-  <si>
-    <t>Built 1950 to 1988</t>
-  </si>
-  <si>
-    <t>Every other verification on file was a visit to one line because something pointed at it (a customer report, a sampling site, a leak on the service, the 2024 ranking), so its shares run high: priced at them the last zone would finish in 2039.</t>
+    <t>Every other verification on file was a visit to one line because something pointed at it (a customer report, a sampling site, a leak on the service, the 2024 ranking), so the lines still unknown are the ones those visits passed over. Priced at the whole-segment shares the last zone would finish in 2038; at the shares across every verification, in 2040.</t>
   </si>
   <si>
     <t>Paid per full replacement completed, 2026 replacement contracts</t>
@@ -712,13 +733,13 @@
         <v>11</v>
       </c>
       <c r="D5" s="4">
-        <v>1670</v>
+        <v>1560</v>
       </c>
       <c r="E5" s="5">
-        <v>23100000</v>
+        <v>21500000</v>
       </c>
       <c r="F5" s="6">
-        <v>23.1</v>
+        <v>21.5</v>
       </c>
       <c r="G5" s="7">
         <v>0.85</v>
@@ -738,16 +759,16 @@
         <v>13</v>
       </c>
       <c r="D6" s="4">
-        <v>2140</v>
+        <v>2020</v>
       </c>
       <c r="E6" s="5">
-        <v>34800000</v>
+        <v>33700000</v>
       </c>
       <c r="F6" s="6">
-        <v>57.9</v>
+        <v>55.2</v>
       </c>
       <c r="G6" s="7">
-        <v>2.14</v>
+        <v>2.17</v>
       </c>
       <c r="H6" s="8">
         <v>2029</v>
@@ -764,16 +785,16 @@
         <v>15</v>
       </c>
       <c r="D7" s="4">
-        <v>1960</v>
+        <v>1830</v>
       </c>
       <c r="E7" s="5">
-        <v>29800000</v>
+        <v>28500000</v>
       </c>
       <c r="F7" s="6">
-        <v>87.7</v>
+        <v>83.7</v>
       </c>
       <c r="G7" s="7">
-        <v>3.24</v>
+        <v>3.3</v>
       </c>
       <c r="H7" s="8">
         <v>2030</v>
@@ -790,16 +811,16 @@
         <v>17</v>
       </c>
       <c r="D8" s="4">
-        <v>1480</v>
+        <v>1420</v>
       </c>
       <c r="E8" s="5">
-        <v>24400000</v>
+        <v>23800000</v>
       </c>
       <c r="F8" s="6">
-        <v>112.1</v>
+        <v>107.5</v>
       </c>
       <c r="G8" s="7">
-        <v>4.14</v>
+        <v>4.23</v>
       </c>
       <c r="H8" s="8">
         <v>2031</v>
@@ -816,16 +837,16 @@
         <v>19</v>
       </c>
       <c r="D9" s="4">
-        <v>1830</v>
+        <v>1730</v>
       </c>
       <c r="E9" s="5">
-        <v>28100000</v>
+        <v>27100000</v>
       </c>
       <c r="F9" s="6">
-        <v>140.2</v>
+        <v>134.6</v>
       </c>
       <c r="G9" s="7">
-        <v>5.17</v>
+        <v>5.3</v>
       </c>
       <c r="H9" s="8">
         <v>2032</v>
@@ -842,16 +863,16 @@
         <v>21</v>
       </c>
       <c r="D10" s="4">
-        <v>1970</v>
+        <v>1840</v>
       </c>
       <c r="E10" s="5">
-        <v>28600000</v>
+        <v>27300000</v>
       </c>
       <c r="F10" s="6">
-        <v>168.9</v>
+        <v>161.9</v>
       </c>
       <c r="G10" s="7">
-        <v>6.23</v>
+        <v>6.37</v>
       </c>
       <c r="H10" s="8">
         <v>2033</v>
@@ -868,16 +889,16 @@
         <v>23</v>
       </c>
       <c r="D11" s="4">
-        <v>1750</v>
+        <v>1640</v>
       </c>
       <c r="E11" s="5">
-        <v>26800000</v>
+        <v>25700000</v>
       </c>
       <c r="F11" s="6">
-        <v>195.7</v>
+        <v>187.6</v>
       </c>
       <c r="G11" s="7">
-        <v>7.22</v>
+        <v>7.38</v>
       </c>
       <c r="H11" s="8">
         <v>2034</v>
@@ -894,19 +915,19 @@
         <v>25</v>
       </c>
       <c r="D12" s="4">
-        <v>930</v>
+        <v>1230</v>
       </c>
       <c r="E12" s="5">
-        <v>15200000</v>
+        <v>19600000</v>
       </c>
       <c r="F12" s="6">
-        <v>210.9</v>
+        <v>207.2</v>
       </c>
       <c r="G12" s="7">
-        <v>7.78</v>
+        <v>8.16</v>
       </c>
       <c r="H12" s="8">
-        <v>2034</v>
+        <v>2035</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -920,16 +941,16 @@
         <v>27</v>
       </c>
       <c r="D13" s="4">
-        <v>1290</v>
+        <v>890</v>
       </c>
       <c r="E13" s="5">
-        <v>20300000</v>
+        <v>14800000</v>
       </c>
       <c r="F13" s="6">
-        <v>231.1</v>
+        <v>222</v>
       </c>
       <c r="G13" s="7">
-        <v>8.529999999999999</v>
+        <v>8.74</v>
       </c>
       <c r="H13" s="8">
         <v>2035</v>
@@ -946,16 +967,16 @@
         <v>29</v>
       </c>
       <c r="D14" s="4">
-        <v>1380</v>
+        <v>1310</v>
       </c>
       <c r="E14" s="5">
-        <v>22100000</v>
+        <v>21400000</v>
       </c>
       <c r="F14" s="6">
-        <v>253.3</v>
+        <v>243.4</v>
       </c>
       <c r="G14" s="7">
-        <v>9.35</v>
+        <v>9.58</v>
       </c>
       <c r="H14" s="8">
         <v>2036</v>
@@ -972,19 +993,19 @@
         <v>31</v>
       </c>
       <c r="D15" s="4">
-        <v>770</v>
+        <v>1040</v>
       </c>
       <c r="E15" s="5">
-        <v>13000000</v>
+        <v>18000000</v>
       </c>
       <c r="F15" s="6">
-        <v>266.2</v>
+        <v>261.4</v>
       </c>
       <c r="G15" s="7">
-        <v>9.82</v>
+        <v>10.29</v>
       </c>
       <c r="H15" s="8">
-        <v>2036</v>
+        <v>2037</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -998,16 +1019,16 @@
         <v>33</v>
       </c>
       <c r="D16" s="10">
-        <v>1080</v>
+        <v>750</v>
       </c>
       <c r="E16" s="11">
-        <v>18400000</v>
+        <v>12700000</v>
       </c>
       <c r="F16" s="12">
-        <v>284.7</v>
+        <v>274.1</v>
       </c>
       <c r="G16" s="13">
-        <v>10.5</v>
+        <v>10.79</v>
       </c>
       <c r="H16" s="14">
         <v>2037</v>
@@ -1022,10 +1043,10 @@
       <c r="D17" s="15"/>
       <c r="E17" s="15"/>
       <c r="F17" s="17">
-        <v>284.7</v>
+        <v>274.1</v>
       </c>
       <c r="G17" s="18">
-        <v>10.5</v>
+        <v>10.79</v>
       </c>
       <c r="H17" s="15"/>
     </row>
@@ -1051,27 +1072,31 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{527D16E0-D497-5745-83E5-630E16E0894B}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>40</v>
       </c>
@@ -1087,61 +1112,170 @@
       <c r="E4" s="3" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="4">
+        <v>12983</v>
+      </c>
+      <c r="C5" s="20">
+        <v>0.556</v>
+      </c>
+      <c r="D5" s="4">
+        <v>7213</v>
+      </c>
+      <c r="E5" s="4">
+        <v>2855</v>
+      </c>
+      <c r="F5" s="4">
+        <v>2177</v>
+      </c>
+      <c r="G5" s="4">
+        <v>10128</v>
+      </c>
+      <c r="H5" s="4">
+        <v>5036</v>
+      </c>
+      <c r="I5" s="20">
+        <v>0.497</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" s="4">
+        <v>10612</v>
+      </c>
+      <c r="C6" s="20">
+        <v>0.316</v>
+      </c>
+      <c r="D6" s="4">
+        <v>3351</v>
+      </c>
+      <c r="E6" s="4">
+        <v>1281</v>
+      </c>
+      <c r="F6" s="4">
+        <v>749</v>
+      </c>
+      <c r="G6" s="4">
+        <v>9331</v>
+      </c>
+      <c r="H6" s="4">
+        <v>2602</v>
+      </c>
+      <c r="I6" s="20">
+        <v>0.279</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="4">
+        <v>13279</v>
+      </c>
+      <c r="C7" s="20">
+        <v>0.083</v>
+      </c>
+      <c r="D7" s="4">
+        <v>1107</v>
+      </c>
+      <c r="E7" s="4">
+        <v>775</v>
+      </c>
+      <c r="F7" s="4">
+        <v>168</v>
+      </c>
+      <c r="G7" s="4">
+        <v>12504</v>
+      </c>
+      <c r="H7" s="4">
+        <v>939</v>
+      </c>
+      <c r="I7" s="20">
+        <v>0.075</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="21" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="32" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B5">
+      <c r="D10" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11">
         <v>792</v>
       </c>
-      <c r="C5">
+      <c r="C11">
         <v>440</v>
       </c>
-      <c r="D5" s="20">
+      <c r="D11" s="20">
         <v>0.556</v>
       </c>
-      <c r="E5" s="20">
-        <v>0.763</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6">
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12">
         <v>304</v>
       </c>
-      <c r="C6">
+      <c r="C12">
         <v>96</v>
       </c>
-      <c r="D6" s="20">
+      <c r="D12" s="20">
         <v>0.316</v>
       </c>
-      <c r="E6" s="20">
-        <v>0.585</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7">
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13">
         <v>168</v>
       </c>
-      <c r="C7">
+      <c r="C13">
         <v>14</v>
       </c>
-      <c r="D7" s="20">
+      <c r="D13" s="20">
         <v>0.083</v>
       </c>
-      <c r="E7" s="20">
-        <v>0.217</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
-        <v>48</v>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="19" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1164,40 +1298,40 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="C5" s="4">
         <v>13890</v>
@@ -1214,10 +1348,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C6" s="4">
         <v>14509</v>
@@ -1234,10 +1368,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B7" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C7" s="4">
         <v>14488</v>
@@ -1254,15 +1388,15 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="C10">
         <v>71</v>
@@ -1279,10 +1413,10 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B11" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C11">
         <v>41</v>
@@ -1299,10 +1433,10 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C12">
         <v>23</v>
@@ -1319,7 +1453,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1340,12 +1474,12 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.25">
@@ -1359,7 +1493,7 @@
         <v>4</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1471,7 +1605,7 @@
         <v>25</v>
       </c>
       <c r="D12" s="4">
-        <v>518</v>
+        <v>626</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1485,7 +1619,7 @@
         <v>27</v>
       </c>
       <c r="D13" s="4">
-        <v>626</v>
+        <v>518</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1513,7 +1647,7 @@
         <v>31</v>
       </c>
       <c r="D15" s="4">
-        <v>368</v>
+        <v>539</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1527,7 +1661,7 @@
         <v>33</v>
       </c>
       <c r="D16" s="4">
-        <v>539</v>
+        <v>368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>